<commit_message>
refactor: cambio en el orden de las columnas y centralizacion de logica
</commit_message>
<xml_diff>
--- a/templates/libros.xlsx
+++ b/templates/libros.xlsx
@@ -18,6 +18,15 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
+    <t xml:space="preserve">Nombre del Socio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° de Socio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha del prestamo</t>
+  </si>
+  <si>
     <t>Autor</t>
   </si>
   <si>
@@ -25,15 +34,6 @@
   </si>
   <si>
     <t xml:space="preserve">N° Inventario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nombre del Socio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° de Socio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fecha del prestamo</t>
   </si>
 </sst>
 </file>
@@ -578,14 +578,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="18.00390625"/>
-    <col customWidth="1" min="2" max="2" width="21.125"/>
-    <col customWidth="1" min="3" max="3" width="19.625"/>
-    <col customWidth="1" min="4" max="4" width="20.375"/>
-    <col customWidth="1" min="5" max="5" width="18.50390625"/>
-    <col customWidth="1" min="6" max="6" width="20.25390625"/>
+    <col customWidth="1" min="1" max="1" width="23.75390625"/>
+    <col customWidth="1" min="2" max="2" width="14.00390625"/>
+    <col customWidth="1" min="3" max="3" width="22.125"/>
+    <col customWidth="1" min="4" max="4" width="18.00390625"/>
+    <col customWidth="1" min="5" max="5" width="21.125"/>
+    <col customWidth="1" min="6" max="6" width="19.625"/>
+    <col customWidth="1" min="7" max="7" width="20.375"/>
+    <col customWidth="1" min="8" max="8" width="18.50390625"/>
+    <col customWidth="1" min="9" max="9" width="20.25390625"/>
   </cols>
   <sheetData>
     <row r="1" ht="15">
@@ -607,7 +610,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
feat: actualiza el template del excel de libros
</commit_message>
<xml_diff>
--- a/templates/libros.xlsx
+++ b/templates/libros.xlsx
@@ -16,24 +16,57 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t xml:space="preserve">Nombre del Socio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° de Socio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fecha del prestamo</t>
-  </si>
-  <si>
-    <t>Autor</t>
-  </si>
-  <si>
-    <t>Titulo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° Inventario</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t xml:space="preserve">Nombre del Socio (1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° de Socio (2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha del prestamo (3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autor (4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titulo (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° Inventario (6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de item (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forma literaria (8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edicion (9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lugar de publicacion (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre Editorial (11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año de publicacion (12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sede (13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sede en tenencia (14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota publica (15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signatura (16)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pais del autor (17)</t>
   </si>
 </sst>
 </file>
@@ -581,14 +614,21 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="23.75390625"/>
-    <col customWidth="1" min="2" max="2" width="14.00390625"/>
-    <col customWidth="1" min="3" max="3" width="22.125"/>
+    <col customWidth="1" min="2" max="2" width="17.50390625"/>
+    <col customWidth="1" min="3" max="3" width="25.50390625"/>
     <col customWidth="1" min="4" max="4" width="18.00390625"/>
     <col customWidth="1" min="5" max="5" width="21.125"/>
     <col customWidth="1" min="6" max="6" width="19.625"/>
-    <col customWidth="1" min="7" max="7" width="20.375"/>
-    <col customWidth="1" min="8" max="8" width="18.50390625"/>
-    <col customWidth="1" min="9" max="9" width="20.25390625"/>
+    <col customWidth="1" min="7" max="7" width="15.50390625"/>
+    <col customWidth="1" min="8" max="8" width="16.75390625"/>
+    <col customWidth="1" min="9" max="9" width="12.625"/>
+    <col customWidth="1" min="10" max="10" width="23.25390625"/>
+    <col customWidth="1" min="11" max="11" width="19.375"/>
+    <col customWidth="1" min="12" max="12" width="19.75390625"/>
+    <col customWidth="1" min="14" max="14" width="20.25390625"/>
+    <col customWidth="1" min="15" max="15" width="15.375"/>
+    <col customWidth="1" min="16" max="16" width="13.75390625"/>
+    <col customWidth="1" min="17" max="17" width="16.00390625"/>
   </cols>
   <sheetData>
     <row r="1" ht="15">
@@ -610,7 +650,39 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="2"/>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
refactor: separa nro de inventario de barCode como datos diferentes
</commit_message>
<xml_diff>
--- a/templates/libros.xlsx
+++ b/templates/libros.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t xml:space="preserve">Nombre del Socio (1)</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t xml:space="preserve">Pais del autor (17)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codigo de barras / ISBN (18)</t>
   </si>
 </sst>
 </file>
@@ -629,6 +632,7 @@
     <col customWidth="1" min="15" max="15" width="15.375"/>
     <col customWidth="1" min="16" max="16" width="13.75390625"/>
     <col customWidth="1" min="17" max="17" width="16.00390625"/>
+    <col customWidth="1" min="18" max="18" width="25.625"/>
   </cols>
   <sheetData>
     <row r="1" ht="15">
@@ -682,6 +686,9 @@
       </c>
       <c r="Q1" t="s">
         <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: agrega el tipo dewey y simplifica el tipo callNumber
</commit_message>
<xml_diff>
--- a/templates/libros.xlsx
+++ b/templates/libros.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">Nombre del Socio (1)</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t xml:space="preserve">Codigo de barras / ISBN (18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CDD (19)</t>
   </si>
 </sst>
 </file>
@@ -690,6 +693,9 @@
       <c r="R1" t="s">
         <v>17</v>
       </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
feat: agrega la propiedad fechaDeIngreso al modelo Libro
</commit_message>
<xml_diff>
--- a/templates/libros.xlsx
+++ b/templates/libros.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">Nombre del Socio (1)</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t xml:space="preserve">CDD (19)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de Ingreso (20)</t>
   </si>
 </sst>
 </file>
@@ -636,6 +639,8 @@
     <col customWidth="1" min="16" max="16" width="13.75390625"/>
     <col customWidth="1" min="17" max="17" width="16.00390625"/>
     <col customWidth="1" min="18" max="18" width="25.625"/>
+    <col customWidth="1" min="19" max="19" width="10.375"/>
+    <col customWidth="1" min="20" max="20" width="20.125"/>
   </cols>
   <sheetData>
     <row r="1" ht="15">
@@ -695,6 +700,9 @@
       </c>
       <c r="S1" t="s">
         <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: agrega LiteraryGenre al modelo de excel
</commit_message>
<xml_diff>
--- a/templates/libros.xlsx
+++ b/templates/libros.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t xml:space="preserve">Nombre del Socio (1)</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t xml:space="preserve">Fecha de Ingreso (20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genero literario (21)</t>
   </si>
 </sst>
 </file>
@@ -641,6 +644,7 @@
     <col customWidth="1" min="18" max="18" width="25.625"/>
     <col customWidth="1" min="19" max="19" width="10.375"/>
     <col customWidth="1" min="20" max="20" width="20.125"/>
+    <col customWidth="1" min="21" max="21" width="18.25390625"/>
   </cols>
   <sheetData>
     <row r="1" ht="15">
@@ -703,6 +707,9 @@
       </c>
       <c r="T1" t="s">
         <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>